<commit_message>
modificari majore dupa primele teste
</commit_message>
<xml_diff>
--- a/test/DentalVoice_Scenarii_Test.xlsx
+++ b/test/DentalVoice_Scenarii_Test.xlsx
@@ -5,23 +5,26 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DentalVoice\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DentalVoice\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD6757A-0E8E-4BA4-88D3-A7D6C24FB545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EEB8725-F602-4F2C-9D31-7B24019FC2FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenarii de Test" sheetId="1" r:id="rId1"/>
     <sheet name="Sumar" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Scenarii de Test'!$A$3:$F$81</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="166">
   <si>
     <t>DentalVoice — Plan de Testare  |  Versiune 1.0  |  Canale: WebBot · WhatsApp</t>
   </si>
@@ -519,15 +522,6 @@
   </si>
   <si>
     <t>Observatii</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Daca incerc sa fac programare manuala, din dashboardul receptiei, si din greseala dau de 2 ori pe "Salveaza Programarea" dupa ce am introdus toate datele, sistemul imi salveaza 2 programari desi eu vreua sa salvez doar o data, am dat din greseala dublu click in loc de click simplu. Asta trebuie evitat.
-2. cand fac programarea manual In continuare apare de 2 ori optiunea "Oricare medic disponibil"
-3. Sa zicem ca lurez la receptie, in dashboardul actual nu pot face mai multe programari intr-un slot orar (desi in configuratia actuala am 3 doctori la clinica de test), deci ar trebui sa pot face intr-un slot orar programari maxim cu numarul de medici configurati. Numarul de medici trebuie sa fie un parametru configurabil.
-4. Daca fac 2 sau mai multe programari in acelasi slot orar (pentru ca am mai multi medici la clinica pot face numar de programari maxim cati medici am) in dashboardul receptiei apare in celula corespunzatoare acelui slot doar "2 programari" sau cate sunt, si nu pot deschide sa vad detaliile fiecarei programare. Ma intereseaza sa vad toate programarile in celula (doar inf generale Nume dr si serviciul oferit) si sa pot deschide fiecare programare in parte pentru a vedea toate detaliile
-5. Pe partea de programare whatsapp, daca aleg data si imi arata sloturile orare, vreau sa am si un buton care sa ma intoarca la alegerea datei cu titlul "Schimba data aleasa" (pe langa toate butoanele cu sloturile orare disponibile)
-6. dupa ce finalizez programarea pe whatsapp si vreau sa imi trimit datele pe email, aleg optiunea sa introduc emailul dar chatul revine la meniul initial, nu imi cere emailul ca sa imi trimita datele programarii
-</t>
   </si>
 </sst>
 </file>
@@ -707,21 +701,21 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1036,20 +1030,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
     </row>
     <row r="2" spans="1:6" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1072,15 +1066,15 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-    </row>
-    <row r="5" spans="1:6" ht="408" x14ac:dyDescent="0.25">
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+    </row>
+    <row r="5" spans="1:6" ht="36" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>1</v>
       </c>
@@ -1091,12 +1085,9 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E5" s="3"/>
-      <c r="F5" s="22" t="s">
-        <v>166</v>
-      </c>
     </row>
     <row r="6" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
@@ -1109,7 +1100,7 @@
         <v>11</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E6" s="6"/>
     </row>
@@ -1124,7 +1115,7 @@
         <v>13</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E7" s="3"/>
     </row>
@@ -1139,7 +1130,7 @@
         <v>15</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E8" s="6"/>
     </row>
@@ -1154,7 +1145,7 @@
         <v>17</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E9" s="3"/>
     </row>
@@ -1169,7 +1160,7 @@
         <v>19</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E10" s="6"/>
     </row>
@@ -1184,7 +1175,7 @@
         <v>21</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E11" s="3"/>
     </row>
@@ -1199,7 +1190,7 @@
         <v>23</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E12" s="6"/>
     </row>
@@ -1214,7 +1205,7 @@
         <v>25</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E13" s="3"/>
     </row>
@@ -1229,7 +1220,7 @@
         <v>27</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E14" s="6"/>
     </row>
@@ -1244,7 +1235,7 @@
         <v>29</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E15" s="3"/>
     </row>
@@ -1259,11 +1250,11 @@
         <v>31</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E16" s="6"/>
     </row>
-    <row r="17" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>13</v>
       </c>
@@ -1274,11 +1265,11 @@
         <v>33</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E17" s="3"/>
     </row>
-    <row r="18" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -1289,11 +1280,11 @@
         <v>35</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E18" s="6"/>
     </row>
-    <row r="19" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>15</v>
       </c>
@@ -1304,11 +1295,11 @@
         <v>37</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -1323,7 +1314,7 @@
       </c>
       <c r="E20" s="6"/>
     </row>
-    <row r="21" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="36" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>17</v>
       </c>
@@ -1334,11 +1325,12 @@
         <v>41</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>9</v>
+        <v>158</v>
       </c>
       <c r="E21" s="3"/>
-    </row>
-    <row r="22" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F21" s="16"/>
+    </row>
+    <row r="22" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -1349,11 +1341,11 @@
         <v>43</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E22" s="6"/>
     </row>
-    <row r="23" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>19</v>
       </c>
@@ -1364,11 +1356,11 @@
         <v>45</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E23" s="3"/>
     </row>
-    <row r="24" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -1383,16 +1375,16 @@
       </c>
       <c r="E24" s="6"/>
     </row>
-    <row r="25" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="18" t="s">
+    <row r="25" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-    </row>
-    <row r="26" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+    </row>
+    <row r="26" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>21</v>
       </c>
@@ -1403,11 +1395,11 @@
         <v>50</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E26" s="3"/>
     </row>
-    <row r="27" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
         <v>22</v>
       </c>
@@ -1418,11 +1410,11 @@
         <v>52</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E27" s="6"/>
     </row>
-    <row r="28" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>23</v>
       </c>
@@ -1433,11 +1425,11 @@
         <v>54</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E28" s="3"/>
     </row>
-    <row r="29" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>24</v>
       </c>
@@ -1448,11 +1440,11 @@
         <v>56</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E29" s="6"/>
     </row>
-    <row r="30" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>25</v>
       </c>
@@ -1463,11 +1455,11 @@
         <v>58</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E30" s="3"/>
     </row>
-    <row r="31" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
         <v>26</v>
       </c>
@@ -1478,11 +1470,11 @@
         <v>60</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E31" s="6"/>
     </row>
-    <row r="32" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>27</v>
       </c>
@@ -1493,7 +1485,7 @@
         <v>62</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E32" s="3"/>
     </row>
@@ -1508,7 +1500,7 @@
         <v>64</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E33" s="6"/>
     </row>
@@ -1523,7 +1515,7 @@
         <v>66</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E34" s="3"/>
     </row>
@@ -1538,7 +1530,7 @@
         <v>68</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E35" s="6"/>
     </row>
@@ -1553,7 +1545,7 @@
         <v>70</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E36" s="3"/>
     </row>
@@ -1568,7 +1560,7 @@
         <v>72</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E37" s="6"/>
     </row>
@@ -1583,7 +1575,7 @@
         <v>74</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E38" s="3"/>
     </row>
@@ -1598,7 +1590,7 @@
         <v>76</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E39" s="6"/>
     </row>
@@ -1613,7 +1605,7 @@
         <v>78</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E40" s="3"/>
     </row>
@@ -1628,18 +1620,18 @@
         <v>80</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E41" s="6"/>
     </row>
     <row r="42" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="18" t="s">
+      <c r="A42" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="B42" s="17"/>
-      <c r="C42" s="17"/>
-      <c r="D42" s="17"/>
-      <c r="E42" s="17"/>
+      <c r="B42" s="18"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="18"/>
     </row>
     <row r="43" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
@@ -1652,7 +1644,7 @@
         <v>83</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E43" s="3"/>
     </row>
@@ -1667,7 +1659,7 @@
         <v>85</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>9</v>
+        <v>158</v>
       </c>
       <c r="E44" s="6"/>
     </row>
@@ -1682,7 +1674,7 @@
         <v>87</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E45" s="3"/>
     </row>
@@ -1697,7 +1689,7 @@
         <v>89</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E46" s="6"/>
     </row>
@@ -1727,18 +1719,18 @@
         <v>93</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E48" s="6"/>
     </row>
     <row r="49" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="18" t="s">
+      <c r="A49" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="B49" s="17"/>
-      <c r="C49" s="17"/>
-      <c r="D49" s="17"/>
-      <c r="E49" s="17"/>
+      <c r="B49" s="18"/>
+      <c r="C49" s="18"/>
+      <c r="D49" s="18"/>
+      <c r="E49" s="18"/>
     </row>
     <row r="50" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
@@ -1751,7 +1743,7 @@
         <v>96</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E50" s="3"/>
     </row>
@@ -1766,7 +1758,7 @@
         <v>98</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E51" s="6"/>
     </row>
@@ -1781,7 +1773,7 @@
         <v>100</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E52" s="3"/>
     </row>
@@ -1796,7 +1788,7 @@
         <v>102</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E53" s="6"/>
     </row>
@@ -1831,13 +1823,13 @@
       <c r="E55" s="6"/>
     </row>
     <row r="56" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="18" t="s">
+      <c r="A56" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="B56" s="17"/>
-      <c r="C56" s="17"/>
-      <c r="D56" s="17"/>
-      <c r="E56" s="17"/>
+      <c r="B56" s="18"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="18"/>
+      <c r="E56" s="18"/>
     </row>
     <row r="57" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
@@ -1865,7 +1857,7 @@
         <v>111</v>
       </c>
       <c r="D58" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E58" s="6"/>
     </row>
@@ -1880,7 +1872,7 @@
         <v>113</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>9</v>
+        <v>158</v>
       </c>
       <c r="E59" s="3"/>
     </row>
@@ -1895,18 +1887,18 @@
         <v>115</v>
       </c>
       <c r="D60" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E60" s="6"/>
     </row>
     <row r="61" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="18" t="s">
+      <c r="A61" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="B61" s="17"/>
-      <c r="C61" s="17"/>
-      <c r="D61" s="17"/>
-      <c r="E61" s="17"/>
+      <c r="B61" s="18"/>
+      <c r="C61" s="18"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="18"/>
     </row>
     <row r="62" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
@@ -1919,7 +1911,7 @@
         <v>118</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E62" s="3"/>
     </row>
@@ -1934,7 +1926,7 @@
         <v>120</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E63" s="6"/>
     </row>
@@ -1949,7 +1941,7 @@
         <v>122</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>9</v>
+        <v>158</v>
       </c>
       <c r="E64" s="3"/>
     </row>
@@ -1964,18 +1956,18 @@
         <v>124</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E65" s="6"/>
     </row>
     <row r="66" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="18" t="s">
+      <c r="A66" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="B66" s="17"/>
-      <c r="C66" s="17"/>
-      <c r="D66" s="17"/>
-      <c r="E66" s="17"/>
+      <c r="B66" s="18"/>
+      <c r="C66" s="18"/>
+      <c r="D66" s="18"/>
+      <c r="E66" s="18"/>
     </row>
     <row r="67" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
@@ -2038,13 +2030,13 @@
       <c r="E70" s="6"/>
     </row>
     <row r="71" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="18" t="s">
+      <c r="A71" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="B71" s="17"/>
-      <c r="C71" s="17"/>
-      <c r="D71" s="17"/>
-      <c r="E71" s="17"/>
+      <c r="B71" s="18"/>
+      <c r="C71" s="18"/>
+      <c r="D71" s="18"/>
+      <c r="E71" s="18"/>
     </row>
     <row r="72" spans="1:5" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
@@ -2117,7 +2109,7 @@
         <v>144</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E76" s="3"/>
     </row>
@@ -2132,7 +2124,7 @@
         <v>146</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="E77" s="6"/>
     </row>
@@ -2197,6 +2189,7 @@
       <c r="E81" s="6"/>
     </row>
   </sheetData>
+  <autoFilter ref="A3:F81" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="10">
     <mergeCell ref="A71:E71"/>
     <mergeCell ref="A49:E49"/>
@@ -2228,14 +2221,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="17"/>
+      <c r="B1" s="18"/>
     </row>
     <row r="2" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17"/>
-      <c r="B2" s="17"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
     </row>
     <row r="3" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
@@ -2251,7 +2244,7 @@
       </c>
       <c r="B4" s="11">
         <f>COUNTIF('Scenarii de Test'!D:D,"✅ OK")</f>
-        <v>1</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -2260,7 +2253,7 @@
       </c>
       <c r="B5" s="13">
         <f>COUNTIF('Scenarii de Test'!D:D,"❌ NOK")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -2269,38 +2262,38 @@
       </c>
       <c r="B6" s="15">
         <f>COUNTIF('Scenarii de Test'!D:D,"⏳ Neptestat")</f>
-        <v>69</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="B8" s="17"/>
+      <c r="B8" s="18"/>
     </row>
     <row r="9" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="B9" s="17"/>
+      <c r="B9" s="18"/>
     </row>
     <row r="10" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="B10" s="17"/>
+      <c r="B10" s="18"/>
     </row>
     <row r="11" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="B11" s="17"/>
+      <c r="B11" s="18"/>
     </row>
     <row r="12" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="B12" s="17"/>
+      <c r="B12" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>